<commit_message>
chore: archive pre-combo-focus state
</commit_message>
<xml_diff>
--- a/public/config/Actions.xlsx
+++ b/public/config/Actions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miko/Code/web-behavior-tree/public/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0743B501-6639-BE43-955E-FF2724FF9C0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D531F6-AFD3-F942-BC29-6E4384D8724E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9940" yWindow="6300" windowWidth="44800" windowHeight="25320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1280" yWindow="600" windowWidth="44800" windowHeight="23820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ActionConfig" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="70">
   <si>
     <t>ActionId</t>
   </si>
@@ -271,12 +271,81 @@
       <t>.mp4</t>
     </r>
   </si>
+  <si>
+    <r>
+      <t>尾巴插地</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="FangSong"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>尾巴充能</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>.mp4</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>尾巴插地放电</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>尾巴充电</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Astaroth_Tail_Ground_Spike_Charged</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF1F2937"/>
@@ -312,6 +381,20 @@
       <color rgb="FF111827"/>
       <name val="FangSong"/>
       <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF111827"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF111827"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -380,7 +463,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -398,6 +481,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -734,7 +820,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -855,317 +941,330 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:4" ht="18" x14ac:dyDescent="0.15">
+      <c r="A9" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" s="5"/>
+    </row>
+    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A10" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B10" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A10" s="5" t="s">
+      <c r="D10" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A11" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B11" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C11" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A11" s="4" t="s">
+      <c r="D11" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A12" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B12" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C12" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A12" s="5" t="s">
+      <c r="D12" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A13" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B13" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A13" s="4" t="s">
+      <c r="D13" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A14" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B14" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A14" s="5" t="s">
+      <c r="D14" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A15" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A15" s="4" t="s">
+      <c r="D15" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A16" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B16" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A16" s="5" t="s">
+      <c r="D16" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A17" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B17" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A17" s="4" t="s">
+      <c r="D17" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A18" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B18" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C18" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A18" s="5" t="s">
+      <c r="D18" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A19" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B19" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D18" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A19" s="4" t="s">
+      <c r="D19" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A20" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B20" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A20" s="5" t="s">
+      <c r="D20" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A21" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B21" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C21" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A21" s="4" t="s">
+      <c r="D21" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A22" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B21" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A22" s="5" t="s">
+      <c r="B22" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A23" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A23" s="4" t="s">
+      <c r="B23" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A24" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A24" s="5" t="s">
+      <c r="B24" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A25" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B24" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A25" s="4" t="s">
+      <c r="B25" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A26" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B25" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A26" s="5" t="s">
+      <c r="B26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A27" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B26" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A27" s="4" t="s">
+      <c r="B27" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A28" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B27" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A28" s="5" t="s">
+      <c r="B28" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A29" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B28" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A29" s="4" t="s">
+      <c r="B29" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A30" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B29" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="15" x14ac:dyDescent="0.15">
-      <c r="A30" s="5" t="s">
+      <c r="B30" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.15">
+      <c r="A31" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B31" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D31" s="5" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:D30" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A2:D31" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: checkpoint before return node
</commit_message>
<xml_diff>
--- a/public/config/Actions.xlsx
+++ b/public/config/Actions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/miko/Code/web-behavior-tree/public/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DE3C10B-FA14-704A-B6C5-64BADF503189}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B91A6B8C-D073-4242-9B48-7F360F6009C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1280" yWindow="600" windowWidth="44800" windowHeight="23820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -169,18 +169,12 @@
     <t>Astaroth_Double_Breath_Charged</t>
   </si>
   <si>
-    <t>二连吐息-头、翅膀充电</t>
-  </si>
-  <si>
     <t>二连吐息-头充电.mp4</t>
   </si>
   <si>
     <t>Astaroth_Head_Double_Swing_Charged</t>
   </si>
   <si>
-    <t>二连甩头-头、翅膀充电</t>
-  </si>
-  <si>
     <t>二连甩头.mp4</t>
   </si>
   <si>
@@ -245,13 +239,77 @@
   </si>
   <si>
     <t>全身放电攻击.mp4</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>二连甩头</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>头</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>二连吐息</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF111827"/>
+        <rFont val="Microsoft YaHei"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>头充电</t>
+    </r>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF1F2937"/>
@@ -293,6 +351,13 @@
       <sz val="11"/>
       <color rgb="FF111827"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF111827"/>
+      <name val="Microsoft YaHei"/>
       <family val="2"/>
       <charset val="134"/>
     </font>
@@ -362,7 +427,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -385,11 +450,25 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF000000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFF4D4F"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -916,95 +995,95 @@
       <c r="A16" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>48</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>49</v>
       </c>
       <c r="D16" s="4"/>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>52</v>
       </c>
       <c r="D17" s="5"/>
     </row>
     <row r="18" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>53</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>55</v>
       </c>
       <c r="D18" s="4"/>
     </row>
     <row r="19" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>56</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="D19" s="5"/>
     </row>
     <row r="20" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="D20" s="4"/>
     </row>
     <row r="21" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>62</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>64</v>
       </c>
       <c r="D21" s="5"/>
     </row>
     <row r="22" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>67</v>
       </c>
       <c r="D22" s="4"/>
     </row>
     <row r="23" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="D23" s="5"/>
     </row>
@@ -1052,19 +1131,29 @@
     </row>
     <row r="31" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>73</v>
       </c>
       <c r="D31" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:D31" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="4" type="noConversion"/>
+  <conditionalFormatting sqref="A3:A1048576">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>AND(A3&lt;&gt;"",COUNTIF($A:$A,A3)&gt;1)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="ActionId 重复" error="A列已有相同 ActionId，请使用唯一 ID。" promptTitle="ActionId 唯一性" prompt="ActionId 需要在 A 列保持唯一。" sqref="A3:A1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
+      <formula1>OR(A3="",COUNTIF($A:$A,A3)=1)</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>